<commit_message>
docs(uat): withdrawal shipped — R-15..R-18 test steps in plan/page/workbook; step count 244
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/uat/ucg-preflight-feedback.xlsx
+++ b/docs/uat/ucg-preflight-feedback.xlsx
@@ -13,8 +13,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Julia Findings'!$A$1:$O$300</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nate Findings'!$A$1:$O$300</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Julia Findings'!$A$1:$O$304</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Nate Findings'!$A$1:$O$304</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1018,7 +1018,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O300"/>
+  <dimension ref="A1:O304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1320,7 +1320,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Admin sends an account invite (#/admin/members), recipient clicks the link</t>
+          <t>Admin sends an account invite: #/admin/members → open a person who has no account → Send account invite. (NOT "+ New Person" — that only creates the profile; A-07-01 was partly this step's wording.) Recipient clicks the link</t>
         </is>
       </c>
       <c r="D10" s="13" t="n"/>
@@ -1874,7 +1874,7 @@
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Simultaneous capacity fill. Set an event cap to a number where you'll collide (e.g. cap 2, you each try to register 2 athletes), then both check out at once</t>
+          <t>⏸ HOLD until the capacity rework ships (your Z-03-02/03 decisions). Then: simultaneous capacity fill — set a cap where you'll collide, both check out at once</t>
         </is>
       </c>
       <c r="D42" s="13" t="n"/>
@@ -4390,27 +4390,38 @@
       </c>
       <c r="D187" s="13" t="n"/>
     </row>
-    <row r="188" ht="20" customHeight="1">
-      <c r="A188" s="9" t="inlineStr">
-        <is>
-          <t>F  -  Finance &amp; admin (Nate + Julia as finance_admin)</t>
-        </is>
-      </c>
+    <row r="188">
+      <c r="A188" s="10" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B188" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C188" s="12" t="inlineStr">
+        <is>
+          <t>NEW (2026-08-24): Withdraw from a UCG-hosted event where your registration cost $0 (100% promo), before lastDateToEdit — the Withdraw button replaces the refund option on My Registrations</t>
+        </is>
+      </c>
+      <c r="D188" s="13" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="inlineStr">
         <is>
-          <t>F-01</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B189" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C189" s="12" t="inlineStr">
         <is>
-          <t>Julia opens #/admin/finance as finance_admin, not admin</t>
+          <t>NEW: Withdraw after lastDateToEdit (any withdrawable registration)</t>
         </is>
       </c>
       <c r="D189" s="13" t="n"/>
@@ -4418,17 +4429,17 @@
     <row r="190">
       <c r="A190" s="10" t="inlineStr">
         <is>
-          <t>F-02</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B190" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C190" s="12" t="inlineStr">
         <is>
-          <t>Summary tab: one line per revenue type with its accounting code</t>
+          <t>NEW: Withdraw from a NON-UCG event (refunds are handled off-platform by the host club)</t>
         </is>
       </c>
       <c r="D190" s="13" t="n"/>
@@ -4436,43 +4447,32 @@
     <row r="191">
       <c r="A191" s="10" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B191" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C191" s="12" t="inlineStr">
         <is>
-          <t>Check the arithmetic by hand against the Stripe Dashboard for one day</t>
+          <t>NEW: Check the refund-vs-withdraw button logic across your registrations</t>
         </is>
       </c>
       <c r="D191" s="13" t="n"/>
     </row>
-    <row r="192">
-      <c r="A192" s="10" t="inlineStr">
-        <is>
-          <t>F-04</t>
-        </is>
-      </c>
-      <c r="B192" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C192" s="12" t="inlineStr">
-        <is>
-          <t>Date-range filter, including the smart defaults (reg-open → event+1wk per event; previous month for the aggregate)</t>
-        </is>
-      </c>
-      <c r="D192" s="13" t="n"/>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="9" t="inlineStr">
+        <is>
+          <t>F  -  Finance &amp; admin (Nate + Julia as finance_admin)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="10" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="B193" s="11" t="inlineStr">
@@ -4482,7 +4482,7 @@
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>Per-event finance dashboard</t>
+          <t>Julia opens #/admin/finance as finance_admin, not admin</t>
         </is>
       </c>
       <c r="D193" s="13" t="n"/>
@@ -4490,7 +4490,7 @@
     <row r="194">
       <c r="A194" s="10" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-02</t>
         </is>
       </c>
       <c r="B194" s="11" t="inlineStr">
@@ -4500,7 +4500,7 @@
       </c>
       <c r="C194" s="12" t="inlineStr">
         <is>
-          <t>Host payout on an event: amount owed + the calculation shown</t>
+          <t>Summary tab: one line per revenue type with its accounting code</t>
         </is>
       </c>
       <c r="D194" s="13" t="n"/>
@@ -4508,7 +4508,7 @@
     <row r="195">
       <c r="A195" s="10" t="inlineStr">
         <is>
-          <t>F-07</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B195" s="11" t="inlineStr">
@@ -4518,7 +4518,7 @@
       </c>
       <c r="C195" s="12" t="inlineStr">
         <is>
-          <t>Enter host payment info (date, check# / PayPal / ACH)</t>
+          <t>Check the arithmetic by hand against the Stripe Dashboard for one day</t>
         </is>
       </c>
       <c r="D195" s="13" t="n"/>
@@ -4526,7 +4526,7 @@
     <row r="196">
       <c r="A196" s="10" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B196" s="11" t="inlineStr">
@@ -4536,7 +4536,7 @@
       </c>
       <c r="C196" s="12" t="inlineStr">
         <is>
-          <t>Invoices/Transactions tab</t>
+          <t>Date-range filter, including the smart defaults (reg-open → event+1wk per event; previous month for the aggregate)</t>
         </is>
       </c>
       <c r="D196" s="13" t="n"/>
@@ -4544,7 +4544,7 @@
     <row r="197">
       <c r="A197" s="10" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B197" s="11" t="inlineStr">
@@ -4554,7 +4554,7 @@
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
-          <t>Click through from a summary line to its transactions</t>
+          <t>Per-event finance dashboard</t>
         </is>
       </c>
       <c r="D197" s="13" t="n"/>
@@ -4562,7 +4562,7 @@
     <row r="198">
       <c r="A198" s="10" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B198" s="11" t="inlineStr">
@@ -4572,7 +4572,7 @@
       </c>
       <c r="C198" s="12" t="inlineStr">
         <is>
-          <t>Export both tabs; open in Excel</t>
+          <t>Host payout on an event: amount owed + the calculation shown</t>
         </is>
       </c>
       <c r="D198" s="13" t="n"/>
@@ -4580,7 +4580,7 @@
     <row r="199">
       <c r="A199" s="10" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>F-07</t>
         </is>
       </c>
       <c r="B199" s="11" t="inlineStr">
@@ -4590,7 +4590,7 @@
       </c>
       <c r="C199" s="12" t="inlineStr">
         <is>
-          <t>Accounting-code management: assign codes to purchase-item types</t>
+          <t>Enter host payment info (date, check# / PayPal / ACH)</t>
         </is>
       </c>
       <c r="D199" s="13" t="n"/>
@@ -4598,7 +4598,7 @@
     <row r="200">
       <c r="A200" s="10" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B200" s="11" t="inlineStr">
@@ -4608,7 +4608,7 @@
       </c>
       <c r="C200" s="12" t="inlineStr">
         <is>
-          <t>#/admin/members: search, open a profile, edit it, export a person's data, delete a person</t>
+          <t>Invoices/Transactions tab</t>
         </is>
       </c>
       <c r="D200" s="13" t="n"/>
@@ -4616,7 +4616,7 @@
     <row r="201">
       <c r="A201" s="10" t="inlineStr">
         <is>
-          <t>F-13</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B201" s="11" t="inlineStr">
@@ -4626,7 +4626,7 @@
       </c>
       <c r="C201" s="12" t="inlineStr">
         <is>
-          <t>#/admin/clubs: create, edit, manage managers</t>
+          <t>Click through from a summary line to its transactions</t>
         </is>
       </c>
       <c r="D201" s="13" t="n"/>
@@ -4634,7 +4634,7 @@
     <row r="202">
       <c r="A202" s="10" t="inlineStr">
         <is>
-          <t>F-14</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B202" s="11" t="inlineStr">
@@ -4644,7 +4644,7 @@
       </c>
       <c r="C202" s="12" t="inlineStr">
         <is>
-          <t>#/admin/league: seasons, levels, regions, promos, waivers, user roles</t>
+          <t>Export both tabs; open in Excel</t>
         </is>
       </c>
       <c r="D202" s="13" t="n"/>
@@ -4652,7 +4652,7 @@
     <row r="203">
       <c r="A203" s="10" t="inlineStr">
         <is>
-          <t>F-15</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B203" s="11" t="inlineStr">
@@ -4662,7 +4662,7 @@
       </c>
       <c r="C203" s="12" t="inlineStr">
         <is>
-          <t>Grant and then revoke a role; have that person refresh</t>
+          <t>Accounting-code management: assign codes to purchase-item types</t>
         </is>
       </c>
       <c r="D203" s="13" t="n"/>
@@ -4670,7 +4670,7 @@
     <row r="204">
       <c r="A204" s="10" t="inlineStr">
         <is>
-          <t>F-16</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B204" s="11" t="inlineStr">
@@ -4680,7 +4680,7 @@
       </c>
       <c r="C204" s="12" t="inlineStr">
         <is>
-          <t>#/admin/errors</t>
+          <t>#/admin/members: search, open a profile, edit it, export a person's data, delete a person</t>
         </is>
       </c>
       <c r="D204" s="13" t="n"/>
@@ -4688,7 +4688,7 @@
     <row r="205">
       <c r="A205" s="10" t="inlineStr">
         <is>
-          <t>F-17</t>
+          <t>F-13</t>
         </is>
       </c>
       <c r="B205" s="11" t="inlineStr">
@@ -4698,7 +4698,7 @@
       </c>
       <c r="C205" s="12" t="inlineStr">
         <is>
-          <t>Payments reconciliation tool</t>
+          <t>#/admin/clubs: create, edit, manage managers</t>
         </is>
       </c>
       <c r="D205" s="13" t="n"/>
@@ -4706,7 +4706,7 @@
     <row r="206">
       <c r="A206" s="10" t="inlineStr">
         <is>
-          <t>F-18</t>
+          <t>F-14</t>
         </is>
       </c>
       <c r="B206" s="11" t="inlineStr">
@@ -4716,32 +4716,43 @@
       </c>
       <c r="C206" s="12" t="inlineStr">
         <is>
-          <t>Manager-access request → review flow</t>
+          <t>#/admin/league: seasons, levels, regions, promos, waivers, user roles</t>
         </is>
       </c>
       <c r="D206" s="13" t="n"/>
     </row>
-    <row r="207" ht="20" customHeight="1">
-      <c r="A207" s="9" t="inlineStr">
-        <is>
-          <t>J  -  Judge &amp; meet day (2 devices required)</t>
-        </is>
-      </c>
+    <row r="207">
+      <c r="A207" s="10" t="inlineStr">
+        <is>
+          <t>F-15</t>
+        </is>
+      </c>
+      <c r="B207" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C207" s="12" t="inlineStr">
+        <is>
+          <t>Grant and then revoke a role; have that person refresh</t>
+        </is>
+      </c>
+      <c r="D207" s="13" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>F-16</t>
         </is>
       </c>
       <c r="B208" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C208" s="12" t="inlineStr">
         <is>
-          <t>Admin/host: generate a judge access code for a live event</t>
+          <t>#/admin/errors</t>
         </is>
       </c>
       <c r="D208" s="13" t="n"/>
@@ -4749,17 +4760,17 @@
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>J-02</t>
+          <t>F-17</t>
         </is>
       </c>
       <c r="B209" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C209" s="12" t="inlineStr">
         <is>
-          <t>On device 2, signed out, scan the QR with the real camera</t>
+          <t>Payments reconciliation tool</t>
         </is>
       </c>
       <c r="D209" s="13" t="n"/>
@@ -4767,43 +4778,32 @@
     <row r="210">
       <c r="A210" s="10" t="inlineStr">
         <is>
-          <t>J-03</t>
+          <t>F-18</t>
         </is>
       </c>
       <c r="B210" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C210" s="12" t="inlineStr">
         <is>
-          <t>On device 2, sign out / clear, then unlock with the 6-digit code</t>
+          <t>Manager-access request → review flow</t>
         </is>
       </c>
       <c r="D210" s="13" t="n"/>
     </row>
-    <row r="211">
-      <c r="A211" s="10" t="inlineStr">
-        <is>
-          <t>J-04</t>
-        </is>
-      </c>
-      <c r="B211" s="11" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="C211" s="12" t="inlineStr">
-        <is>
-          <t>Enter a wrong 6-digit code</t>
-        </is>
-      </c>
-      <c r="D211" s="13" t="n"/>
+    <row r="211" ht="20" customHeight="1">
+      <c r="A211" s="9" t="inlineStr">
+        <is>
+          <t>J  -  Judge &amp; meet day (2 devices required)</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="10" t="inlineStr">
         <is>
-          <t>J-05</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B212" s="11" t="inlineStr">
@@ -4813,7 +4813,7 @@
       </c>
       <c r="C212" s="12" t="inlineStr">
         <is>
-          <t>After being rate-limited, unlock with the URL/QR token instead</t>
+          <t>Admin/host: generate a judge access code for a live event</t>
         </is>
       </c>
       <c r="D212" s="13" t="n"/>
@@ -4821,7 +4821,7 @@
     <row r="213">
       <c r="A213" s="10" t="inlineStr">
         <is>
-          <t>J-06</t>
+          <t>J-02</t>
         </is>
       </c>
       <c r="B213" s="11" t="inlineStr">
@@ -4831,7 +4831,7 @@
       </c>
       <c r="C213" s="12" t="inlineStr">
         <is>
-          <t>After a successful unlock, try a few bad codes again</t>
+          <t>On device 2, signed out, scan the QR with the real camera</t>
         </is>
       </c>
       <c r="D213" s="13" t="n"/>
@@ -4839,7 +4839,7 @@
     <row r="214">
       <c r="A214" s="10" t="inlineStr">
         <is>
-          <t>J-07</t>
+          <t>J-03</t>
         </is>
       </c>
       <c r="B214" s="11" t="inlineStr">
@@ -4849,7 +4849,7 @@
       </c>
       <c r="C214" s="12" t="inlineStr">
         <is>
-          <t>Enter a real score from the anonymous device</t>
+          <t>On device 2, sign out / clear, then unlock with the 6-digit code</t>
         </is>
       </c>
       <c r="D214" s="13" t="n"/>
@@ -4857,7 +4857,7 @@
     <row r="215">
       <c r="A215" s="10" t="inlineStr">
         <is>
-          <t>J-08</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B215" s="11" t="inlineStr">
@@ -4867,7 +4867,7 @@
       </c>
       <c r="C215" s="12" t="inlineStr">
         <is>
-          <t>Watch that score appear on device 1 without refreshing</t>
+          <t>Enter a wrong 6-digit code</t>
         </is>
       </c>
       <c r="D215" s="13" t="n"/>
@@ -4875,7 +4875,7 @@
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
         <is>
-          <t>J-09</t>
+          <t>J-05</t>
         </is>
       </c>
       <c r="B216" s="11" t="inlineStr">
@@ -4885,7 +4885,7 @@
       </c>
       <c r="C216" s="12" t="inlineStr">
         <is>
-          <t>Use the calculator entry mode</t>
+          <t>After being rate-limited, unlock with the URL/QR token instead</t>
         </is>
       </c>
       <c r="D216" s="13" t="n"/>
@@ -4893,7 +4893,7 @@
     <row r="217">
       <c r="A217" s="10" t="inlineStr">
         <is>
-          <t>J-10</t>
+          <t>J-06</t>
         </is>
       </c>
       <c r="B217" s="11" t="inlineStr">
@@ -4903,7 +4903,7 @@
       </c>
       <c r="C217" s="12" t="inlineStr">
         <is>
-          <t>Use the simple entry mode</t>
+          <t>After a successful unlock, try a few bad codes again</t>
         </is>
       </c>
       <c r="D217" s="13" t="n"/>
@@ -4911,7 +4911,7 @@
     <row r="218">
       <c r="A218" s="10" t="inlineStr">
         <is>
-          <t>J-11</t>
+          <t>J-07</t>
         </is>
       </c>
       <c r="B218" s="11" t="inlineStr">
@@ -4921,7 +4921,7 @@
       </c>
       <c r="C218" s="12" t="inlineStr">
         <is>
-          <t>Event configured for a 2-judge panel</t>
+          <t>Enter a real score from the anonymous device</t>
         </is>
       </c>
       <c r="D218" s="13" t="n"/>
@@ -4929,7 +4929,7 @@
     <row r="219">
       <c r="A219" s="10" t="inlineStr">
         <is>
-          <t>J-12</t>
+          <t>J-08</t>
         </is>
       </c>
       <c r="B219" s="11" t="inlineStr">
@@ -4939,7 +4939,7 @@
       </c>
       <c r="C219" s="12" t="inlineStr">
         <is>
-          <t>Enter scores for each discipline you support (MAG, WAG, T&amp;T, and the specialty calculators)</t>
+          <t>Watch that score appear on device 1 without refreshing</t>
         </is>
       </c>
       <c r="D219" s="13" t="n"/>
@@ -4947,7 +4947,7 @@
     <row r="220">
       <c r="A220" s="10" t="inlineStr">
         <is>
-          <t>J-13</t>
+          <t>J-09</t>
         </is>
       </c>
       <c r="B220" s="11" t="inlineStr">
@@ -4957,7 +4957,7 @@
       </c>
       <c r="C220" s="12" t="inlineStr">
         <is>
-          <t>Edit a posted score</t>
+          <t>Use the calculator entry mode</t>
         </is>
       </c>
       <c r="D220" s="13" t="n"/>
@@ -4965,7 +4965,7 @@
     <row r="221">
       <c r="A221" s="10" t="inlineStr">
         <is>
-          <t>J-14</t>
+          <t>J-10</t>
         </is>
       </c>
       <c r="B221" s="11" t="inlineStr">
@@ -4975,7 +4975,7 @@
       </c>
       <c r="C221" s="12" t="inlineStr">
         <is>
-          <t>Open a score detail page</t>
+          <t>Use the simple entry mode</t>
         </is>
       </c>
       <c r="D221" s="13" t="n"/>
@@ -4983,7 +4983,7 @@
     <row r="222">
       <c r="A222" s="10" t="inlineStr">
         <is>
-          <t>J-15</t>
+          <t>J-11</t>
         </is>
       </c>
       <c r="B222" s="11" t="inlineStr">
@@ -4993,7 +4993,7 @@
       </c>
       <c r="C222" s="12" t="inlineStr">
         <is>
-          <t>Try score entry on a device with no unlock and no privileged account</t>
+          <t>Event configured for a 2-judge panel</t>
         </is>
       </c>
       <c r="D222" s="13" t="n"/>
@@ -5001,7 +5001,7 @@
     <row r="223">
       <c r="A223" s="10" t="inlineStr">
         <is>
-          <t>J-16</t>
+          <t>J-12</t>
         </is>
       </c>
       <c r="B223" s="11" t="inlineStr">
@@ -5011,7 +5011,7 @@
       </c>
       <c r="C223" s="12" t="inlineStr">
         <is>
-          <t>Judge on a phone in landscape, one-handed, on venue-grade wifi</t>
+          <t>Enter scores for each discipline you support (MAG, WAG, T&amp;T, and the specialty calculators)</t>
         </is>
       </c>
       <c r="D223" s="13" t="n"/>
@@ -5019,7 +5019,7 @@
     <row r="224">
       <c r="A224" s="10" t="inlineStr">
         <is>
-          <t>J-17</t>
+          <t>J-13</t>
         </is>
       </c>
       <c r="B224" s="11" t="inlineStr">
@@ -5029,32 +5029,43 @@
       </c>
       <c r="C224" s="12" t="inlineStr">
         <is>
-          <t>Turn wifi off mid-entry, then back on</t>
+          <t>Edit a posted score</t>
         </is>
       </c>
       <c r="D224" s="13" t="n"/>
     </row>
-    <row r="225" ht="20" customHeight="1">
-      <c r="A225" s="9" t="inlineStr">
-        <is>
-          <t>X  -  Public &amp; anonymous surfaces</t>
-        </is>
-      </c>
+    <row r="225">
+      <c r="A225" s="10" t="inlineStr">
+        <is>
+          <t>J-14</t>
+        </is>
+      </c>
+      <c r="B225" s="11" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C225" s="12" t="inlineStr">
+        <is>
+          <t>Open a score detail page</t>
+        </is>
+      </c>
+      <c r="D225" s="13" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="10" t="inlineStr">
         <is>
-          <t>X-01</t>
+          <t>J-15</t>
         </is>
       </c>
       <c r="B226" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C226" s="12" t="inlineStr">
         <is>
-          <t>Public Results index and an event's results</t>
+          <t>Try score entry on a device with no unlock and no privileged account</t>
         </is>
       </c>
       <c r="D226" s="13" t="n"/>
@@ -5062,17 +5073,17 @@
     <row r="227">
       <c r="A227" s="10" t="inlineStr">
         <is>
-          <t>X-02</t>
+          <t>J-16</t>
         </is>
       </c>
       <c r="B227" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C227" s="12" t="inlineStr">
         <is>
-          <t>Results for an event with scores across multiple sessions</t>
+          <t>Judge on a phone in both portrait and landscape, one-handed, on venue-grade wifi — every control reachable in portrait without sideways scrolling (Nate's Z-06 finding)</t>
         </is>
       </c>
       <c r="D227" s="13" t="n"/>
@@ -5080,43 +5091,32 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>J-17</t>
         </is>
       </c>
       <c r="B228" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C228" s="12" t="inlineStr">
         <is>
-          <t>Results for an event where some registrations have no session assigned</t>
+          <t>Turn wifi off mid-entry, then back on</t>
         </is>
       </c>
       <c r="D228" s="13" t="n"/>
     </row>
-    <row r="229">
-      <c r="A229" s="10" t="inlineStr">
-        <is>
-          <t>X-04</t>
-        </is>
-      </c>
-      <c r="B229" s="11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C229" s="12" t="inlineStr">
-        <is>
-          <t>Public Events list and an event detail page</t>
-        </is>
-      </c>
-      <c r="D229" s="13" t="n"/>
+    <row r="229" ht="20" customHeight="1">
+      <c r="A229" s="9" t="inlineStr">
+        <is>
+          <t>X  -  Public &amp; anonymous surfaces</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>X-05</t>
+          <t>X-01</t>
         </is>
       </c>
       <c r="B230" s="11" t="inlineStr">
@@ -5126,7 +5126,7 @@
       </c>
       <c r="C230" s="12" t="inlineStr">
         <is>
-          <t>Home page while signed out</t>
+          <t>Public Results index and an event's results</t>
         </is>
       </c>
       <c r="D230" s="13" t="n"/>
@@ -5134,7 +5134,7 @@
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
         <is>
-          <t>X-06</t>
+          <t>X-02</t>
         </is>
       </c>
       <c r="B231" s="11" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="C231" s="12" t="inlineStr">
         <is>
-          <t>Try #/me, #/cart, #/admin/members while signed out</t>
+          <t>Results for an event with scores across multiple sessions</t>
         </is>
       </c>
       <c r="D231" s="13" t="n"/>
@@ -5152,7 +5152,7 @@
     <row r="232">
       <c r="A232" s="10" t="inlineStr">
         <is>
-          <t>X-07</t>
+          <t>X-03</t>
         </is>
       </c>
       <c r="B232" s="11" t="inlineStr">
@@ -5162,7 +5162,7 @@
       </c>
       <c r="C232" s="12" t="inlineStr">
         <is>
-          <t>Open a judge access URL you weren't given (guess a token)</t>
+          <t>Results for an event where some registrations have no session assigned</t>
         </is>
       </c>
       <c r="D232" s="13" t="n"/>
@@ -5170,7 +5170,7 @@
     <row r="233">
       <c r="A233" s="10" t="inlineStr">
         <is>
-          <t>X-08</t>
+          <t>X-04</t>
         </is>
       </c>
       <c r="B233" s="11" t="inlineStr">
@@ -5180,7 +5180,7 @@
       </c>
       <c r="C233" s="12" t="inlineStr">
         <is>
-          <t>Share an event link to yourself via text/Slack and open it from there</t>
+          <t>Public Events list and an event detail page</t>
         </is>
       </c>
       <c r="D233" s="13" t="n"/>
@@ -5188,7 +5188,7 @@
     <row r="234">
       <c r="A234" s="10" t="inlineStr">
         <is>
-          <t>X-09</t>
+          <t>X-05</t>
         </is>
       </c>
       <c r="B234" s="11" t="inlineStr">
@@ -5198,32 +5198,43 @@
       </c>
       <c r="C234" s="12" t="inlineStr">
         <is>
-          <t>Public pages on a phone</t>
+          <t>Home page while signed out</t>
         </is>
       </c>
       <c r="D234" s="13" t="n"/>
     </row>
-    <row r="235" ht="20" customHeight="1">
-      <c r="A235" s="9" t="inlineStr">
-        <is>
-          <t>D  -  Devices, responsive &amp; PWA</t>
-        </is>
-      </c>
+    <row r="235">
+      <c r="A235" s="10" t="inlineStr">
+        <is>
+          <t>X-06</t>
+        </is>
+      </c>
+      <c r="B235" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C235" s="12" t="inlineStr">
+        <is>
+          <t>Try #/me, #/cart, #/admin/members while signed out</t>
+        </is>
+      </c>
+      <c r="D235" s="13" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="10" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>X-07</t>
         </is>
       </c>
       <c r="B236" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C236" s="12" t="inlineStr">
         <is>
-          <t>Full pass on an iPhone (Safari) — sign in, register, cart, profile</t>
+          <t>Open a judge access URL you weren't given (guess a token)</t>
         </is>
       </c>
       <c r="D236" s="13" t="n"/>
@@ -5231,17 +5242,17 @@
     <row r="237">
       <c r="A237" s="10" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>X-08</t>
         </is>
       </c>
       <c r="B237" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C237" s="12" t="inlineStr">
         <is>
-          <t>Full pass on an Android (Chrome)</t>
+          <t>Share an event link to yourself via text/Slack and open it from there</t>
         </is>
       </c>
       <c r="D237" s="13" t="n"/>
@@ -5249,43 +5260,32 @@
     <row r="238">
       <c r="A238" s="10" t="inlineStr">
         <is>
-          <t>D-03</t>
+          <t>X-09</t>
         </is>
       </c>
       <c r="B238" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C238" s="12" t="inlineStr">
         <is>
-          <t>Tablet, both orientations</t>
+          <t>Public pages on a phone</t>
         </is>
       </c>
       <c r="D238" s="13" t="n"/>
     </row>
-    <row r="239">
-      <c r="A239" s="10" t="inlineStr">
-        <is>
-          <t>D-04</t>
-        </is>
-      </c>
-      <c r="B239" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C239" s="12" t="inlineStr">
-        <is>
-          <t>The mobile nav drawer: open, navigate, close</t>
-        </is>
-      </c>
-      <c r="D239" s="13" t="n"/>
+    <row r="239" ht="20" customHeight="1">
+      <c r="A239" s="9" t="inlineStr">
+        <is>
+          <t>D  -  Devices, responsive &amp; PWA</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="10" t="inlineStr">
         <is>
-          <t>D-05</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B240" s="11" t="inlineStr">
@@ -5295,7 +5295,7 @@
       </c>
       <c r="C240" s="12" t="inlineStr">
         <is>
-          <t>Every modal on a phone — registration popup, refund dialog, report-a-problem</t>
+          <t>Full pass on an iPhone (Safari) — sign in, register, cart, profile</t>
         </is>
       </c>
       <c r="D240" s="13" t="n"/>
@@ -5303,7 +5303,7 @@
     <row r="241">
       <c r="A241" s="10" t="inlineStr">
         <is>
-          <t>D-06</t>
+          <t>D-02</t>
         </is>
       </c>
       <c r="B241" s="11" t="inlineStr">
@@ -5313,7 +5313,7 @@
       </c>
       <c r="C241" s="12" t="inlineStr">
         <is>
-          <t>Wide tables on a phone — admin members, finance transactions, host summary</t>
+          <t>Full pass on an Android (Chrome)</t>
         </is>
       </c>
       <c r="D241" s="13" t="n"/>
@@ -5321,7 +5321,7 @@
     <row r="242">
       <c r="A242" s="10" t="inlineStr">
         <is>
-          <t>D-07</t>
+          <t>D-03</t>
         </is>
       </c>
       <c r="B242" s="11" t="inlineStr">
@@ -5331,7 +5331,7 @@
       </c>
       <c r="C242" s="12" t="inlineStr">
         <is>
-          <t>Install the PWA ("Add to Home Screen") on iOS and Android</t>
+          <t>Tablet, both orientations</t>
         </is>
       </c>
       <c r="D242" s="13" t="n"/>
@@ -5339,7 +5339,7 @@
     <row r="243">
       <c r="A243" s="10" t="inlineStr">
         <is>
-          <t>D-08</t>
+          <t>D-04</t>
         </is>
       </c>
       <c r="B243" s="11" t="inlineStr">
@@ -5349,7 +5349,7 @@
       </c>
       <c r="C243" s="12" t="inlineStr">
         <is>
-          <t>Use the installed PWA for a full registration flow</t>
+          <t>The mobile nav drawer: open, navigate, close</t>
         </is>
       </c>
       <c r="D243" s="13" t="n"/>
@@ -5357,7 +5357,7 @@
     <row r="244">
       <c r="A244" s="10" t="inlineStr">
         <is>
-          <t>D-09</t>
+          <t>D-05</t>
         </is>
       </c>
       <c r="B244" s="11" t="inlineStr">
@@ -5367,7 +5367,7 @@
       </c>
       <c r="C244" s="12" t="inlineStr">
         <is>
-          <t>PWA update path: with the PWA installed, wait for the next deploy, then reopen it</t>
+          <t>Every modal on a phone — registration popup, refund dialog, report-a-problem</t>
         </is>
       </c>
       <c r="D244" s="13" t="n"/>
@@ -5375,7 +5375,7 @@
     <row r="245">
       <c r="A245" s="10" t="inlineStr">
         <is>
-          <t>D-10</t>
+          <t>D-06</t>
         </is>
       </c>
       <c r="B245" s="11" t="inlineStr">
@@ -5385,7 +5385,7 @@
       </c>
       <c r="C245" s="12" t="inlineStr">
         <is>
-          <t>Dark mode (OS-level) on a few pages</t>
+          <t>Wide tables on a phone — admin members, finance transactions, host summary</t>
         </is>
       </c>
       <c r="D245" s="13" t="n"/>
@@ -5393,7 +5393,7 @@
     <row r="246">
       <c r="A246" s="10" t="inlineStr">
         <is>
-          <t>D-11</t>
+          <t>D-07</t>
         </is>
       </c>
       <c r="B246" s="11" t="inlineStr">
@@ -5403,7 +5403,7 @@
       </c>
       <c r="C246" s="12" t="inlineStr">
         <is>
-          <t>Browser zoom to 200% on desktop</t>
+          <t>Install the PWA ("Add to Home Screen") on iOS and Android</t>
         </is>
       </c>
       <c r="D246" s="13" t="n"/>
@@ -5411,7 +5411,7 @@
     <row r="247">
       <c r="A247" s="10" t="inlineStr">
         <is>
-          <t>D-12</t>
+          <t>D-08</t>
         </is>
       </c>
       <c r="B247" s="11" t="inlineStr">
@@ -5421,7 +5421,7 @@
       </c>
       <c r="C247" s="12" t="inlineStr">
         <is>
-          <t>Rotate the phone mid-form</t>
+          <t>Use the installed PWA for a full registration flow</t>
         </is>
       </c>
       <c r="D247" s="13" t="n"/>
@@ -5429,7 +5429,7 @@
     <row r="248">
       <c r="A248" s="10" t="inlineStr">
         <is>
-          <t>D-13</t>
+          <t>D-09</t>
         </is>
       </c>
       <c r="B248" s="11" t="inlineStr">
@@ -5439,32 +5439,43 @@
       </c>
       <c r="C248" s="12" t="inlineStr">
         <is>
-          <t>Firefox and Edge, one flow each</t>
+          <t>PWA update path: with the PWA installed, wait for the next deploy, then reopen it</t>
         </is>
       </c>
       <c r="D248" s="13" t="n"/>
     </row>
-    <row r="249" ht="20" customHeight="1">
-      <c r="A249" s="9" t="inlineStr">
-        <is>
-          <t>Y  -  Keyboard &amp; accessibility (Nate)</t>
-        </is>
-      </c>
+    <row r="249">
+      <c r="A249" s="10" t="inlineStr">
+        <is>
+          <t>D-10</t>
+        </is>
+      </c>
+      <c r="B249" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C249" s="12" t="inlineStr">
+        <is>
+          <t>Dark mode (OS-level) on a few pages</t>
+        </is>
+      </c>
+      <c r="D249" s="13" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="10" t="inlineStr">
         <is>
-          <t>Y-01</t>
+          <t>D-11</t>
         </is>
       </c>
       <c r="B250" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C250" s="12" t="inlineStr">
         <is>
-          <t>Unplug the mouse. Complete one full registration + checkout using only the keyboard</t>
+          <t>Browser zoom to 200% on desktop</t>
         </is>
       </c>
       <c r="D250" s="13" t="n"/>
@@ -5472,17 +5483,17 @@
     <row r="251">
       <c r="A251" s="10" t="inlineStr">
         <is>
-          <t>Y-02</t>
+          <t>D-12</t>
         </is>
       </c>
       <c r="B251" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C251" s="12" t="inlineStr">
         <is>
-          <t>Tab through a page — is the focus ring always visible?</t>
+          <t>Rotate the phone mid-form</t>
         </is>
       </c>
       <c r="D251" s="13" t="n"/>
@@ -5490,43 +5501,32 @@
     <row r="252">
       <c r="A252" s="10" t="inlineStr">
         <is>
-          <t>Y-03</t>
+          <t>D-13</t>
         </is>
       </c>
       <c r="B252" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C252" s="12" t="inlineStr">
         <is>
-          <t>Press Enter and Space on buttons — especially Details/Hide toggles, the judge score stepper, Copy-link buttons</t>
+          <t>Firefox and Edge, one flow each</t>
         </is>
       </c>
       <c r="D252" s="13" t="n"/>
     </row>
-    <row r="253">
-      <c r="A253" s="10" t="inlineStr">
-        <is>
-          <t>Y-04</t>
-        </is>
-      </c>
-      <c r="B253" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C253" s="12" t="inlineStr">
-        <is>
-          <t>Open a modal, then press Tab repeatedly</t>
-        </is>
-      </c>
-      <c r="D253" s="13" t="n"/>
+    <row r="253" ht="20" customHeight="1">
+      <c r="A253" s="9" t="inlineStr">
+        <is>
+          <t>Y  -  Keyboard &amp; accessibility (Nate)</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="10" t="inlineStr">
         <is>
-          <t>Y-05</t>
+          <t>Y-01</t>
         </is>
       </c>
       <c r="B254" s="11" t="inlineStr">
@@ -5536,7 +5536,7 @@
       </c>
       <c r="C254" s="12" t="inlineStr">
         <is>
-          <t>Press Escape in a modal with unsaved changes</t>
+          <t>Unplug the mouse. Complete one full registration + checkout using only the keyboard</t>
         </is>
       </c>
       <c r="D254" s="13" t="n"/>
@@ -5544,7 +5544,7 @@
     <row r="255">
       <c r="A255" s="10" t="inlineStr">
         <is>
-          <t>Y-06</t>
+          <t>Y-02</t>
         </is>
       </c>
       <c r="B255" s="11" t="inlineStr">
@@ -5554,7 +5554,7 @@
       </c>
       <c r="C255" s="12" t="inlineStr">
         <is>
-          <t>Press Escape with two dialogs stacked</t>
+          <t>Tab through a page — is the focus ring always visible?</t>
         </is>
       </c>
       <c r="D255" s="13" t="n"/>
@@ -5562,7 +5562,7 @@
     <row r="256">
       <c r="A256" s="10" t="inlineStr">
         <is>
-          <t>Y-07</t>
+          <t>Y-03</t>
         </is>
       </c>
       <c r="B256" s="11" t="inlineStr">
@@ -5572,7 +5572,7 @@
       </c>
       <c r="C256" s="12" t="inlineStr">
         <is>
-          <t>Close a modal</t>
+          <t>Press Enter and Space on buttons — especially Details/Hide toggles, the judge score stepper, Copy-link buttons</t>
         </is>
       </c>
       <c r="D256" s="13" t="n"/>
@@ -5580,7 +5580,7 @@
     <row r="257">
       <c r="A257" s="10" t="inlineStr">
         <is>
-          <t>Y-08</t>
+          <t>Y-04</t>
         </is>
       </c>
       <c r="B257" s="11" t="inlineStr">
@@ -5590,7 +5590,7 @@
       </c>
       <c r="C257" s="12" t="inlineStr">
         <is>
-          <t>Tab order on a long form (Profile)</t>
+          <t>Open a modal, then press Tab repeatedly</t>
         </is>
       </c>
       <c r="D257" s="13" t="n"/>
@@ -5598,7 +5598,7 @@
     <row r="258">
       <c r="A258" s="10" t="inlineStr">
         <is>
-          <t>Y-09</t>
+          <t>Y-05</t>
         </is>
       </c>
       <c r="B258" s="11" t="inlineStr">
@@ -5608,7 +5608,7 @@
       </c>
       <c r="C258" s="12" t="inlineStr">
         <is>
-          <t>Squint-test every screen for low-contrast text</t>
+          <t>Press Escape in a modal with unsaved changes</t>
         </is>
       </c>
       <c r="D258" s="13" t="n"/>
@@ -5616,43 +5616,99 @@
     <row r="259">
       <c r="A259" s="10" t="inlineStr">
         <is>
+          <t>Y-06</t>
+        </is>
+      </c>
+      <c r="B259" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C259" s="12" t="inlineStr">
+        <is>
+          <t>Press Escape with two dialogs stacked</t>
+        </is>
+      </c>
+      <c r="D259" s="13" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="inlineStr">
+        <is>
+          <t>Y-07</t>
+        </is>
+      </c>
+      <c r="B260" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="inlineStr">
+        <is>
+          <t>Close a modal</t>
+        </is>
+      </c>
+      <c r="D260" s="13" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="10" t="inlineStr">
+        <is>
+          <t>Y-08</t>
+        </is>
+      </c>
+      <c r="B261" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C261" s="12" t="inlineStr">
+        <is>
+          <t>Tab order on a long form (Profile)</t>
+        </is>
+      </c>
+      <c r="D261" s="13" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="inlineStr">
+        <is>
+          <t>Y-09</t>
+        </is>
+      </c>
+      <c r="B262" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="inlineStr">
+        <is>
+          <t>Squint-test every screen for low-contrast text</t>
+        </is>
+      </c>
+      <c r="D262" s="13" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="10" t="inlineStr">
+        <is>
           <t>Y-10</t>
         </is>
       </c>
-      <c r="B259" s="11" t="inlineStr">
+      <c r="B263" s="11" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C259" s="12" t="inlineStr">
+      <c r="C263" s="12" t="inlineStr">
         <is>
           <t>If you have VoiceOver/Narrator, skim the Profile page</t>
         </is>
       </c>
-      <c r="D259" s="13" t="n"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="14" t="inlineStr">
+      <c r="D263" s="13" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="14" t="inlineStr">
         <is>
           <t>EXTRA  -  findings not tied to a step (use e.g. M-X-01)</t>
         </is>
       </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="13" t="n"/>
-      <c r="D261" s="13" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="13" t="n"/>
-      <c r="D262" s="13" t="n"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="13" t="n"/>
-      <c r="D263" s="13" t="n"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="13" t="n"/>
-      <c r="D264" s="13" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="13" t="n"/>
@@ -5798,39 +5854,55 @@
       <c r="A300" s="13" t="n"/>
       <c r="D300" s="13" t="n"/>
     </row>
+    <row r="301">
+      <c r="A301" s="13" t="n"/>
+      <c r="D301" s="13" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="13" t="n"/>
+      <c r="D302" s="13" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="13" t="n"/>
+      <c r="D303" s="13" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="13" t="n"/>
+      <c r="D304" s="13" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O300"/>
+  <autoFilter ref="A1:O304"/>
   <mergeCells count="18">
+    <mergeCell ref="A239:O239"/>
     <mergeCell ref="A81:O81"/>
-    <mergeCell ref="A235:O235"/>
     <mergeCell ref="A105:O105"/>
     <mergeCell ref="A121:O121"/>
-    <mergeCell ref="A260:O260"/>
     <mergeCell ref="A60:O60"/>
-    <mergeCell ref="A207:O207"/>
-    <mergeCell ref="A225:O225"/>
+    <mergeCell ref="A264:O264"/>
+    <mergeCell ref="A253:O253"/>
     <mergeCell ref="A94:O94"/>
     <mergeCell ref="A46:O46"/>
     <mergeCell ref="A155:O155"/>
-    <mergeCell ref="A188:O188"/>
-    <mergeCell ref="A249:O249"/>
+    <mergeCell ref="A211:O211"/>
+    <mergeCell ref="A229:O229"/>
     <mergeCell ref="A135:O135"/>
     <mergeCell ref="A173:O173"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A192:O192"/>
     <mergeCell ref="A39:O39"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="D2:D300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,MISSING,UNCLEAR,BLOCKED,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S1,S2,S3,S4,Q,D"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>
@@ -5844,7 +5916,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O300"/>
+  <dimension ref="A1:O304"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -6146,7 +6218,7 @@
       </c>
       <c r="C10" s="12" t="inlineStr">
         <is>
-          <t>Admin sends an account invite (#/admin/members), recipient clicks the link</t>
+          <t>Admin sends an account invite: #/admin/members → open a person who has no account → Send account invite. (NOT "+ New Person" — that only creates the profile; A-07-01 was partly this step's wording.) Recipient clicks the link</t>
         </is>
       </c>
       <c r="D10" s="13" t="n"/>
@@ -6700,7 +6772,7 @@
       </c>
       <c r="C42" s="12" t="inlineStr">
         <is>
-          <t>Simultaneous capacity fill. Set an event cap to a number where you'll collide (e.g. cap 2, you each try to register 2 athletes), then both check out at once</t>
+          <t>⏸ HOLD until the capacity rework ships (your Z-03-02/03 decisions). Then: simultaneous capacity fill — set a cap where you'll collide, both check out at once</t>
         </is>
       </c>
       <c r="D42" s="13" t="n"/>
@@ -9216,27 +9288,38 @@
       </c>
       <c r="D187" s="13" t="n"/>
     </row>
-    <row r="188" ht="20" customHeight="1">
-      <c r="A188" s="9" t="inlineStr">
-        <is>
-          <t>F  -  Finance &amp; admin (Nate + Julia as finance_admin)</t>
-        </is>
-      </c>
+    <row r="188">
+      <c r="A188" s="10" t="inlineStr">
+        <is>
+          <t>R-15</t>
+        </is>
+      </c>
+      <c r="B188" s="11" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="C188" s="12" t="inlineStr">
+        <is>
+          <t>NEW (2026-08-24): Withdraw from a UCG-hosted event where your registration cost $0 (100% promo), before lastDateToEdit — the Withdraw button replaces the refund option on My Registrations</t>
+        </is>
+      </c>
+      <c r="D188" s="13" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="10" t="inlineStr">
         <is>
-          <t>F-01</t>
+          <t>R-16</t>
         </is>
       </c>
       <c r="B189" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C189" s="12" t="inlineStr">
         <is>
-          <t>Julia opens #/admin/finance as finance_admin, not admin</t>
+          <t>NEW: Withdraw after lastDateToEdit (any withdrawable registration)</t>
         </is>
       </c>
       <c r="D189" s="13" t="n"/>
@@ -9244,17 +9327,17 @@
     <row r="190">
       <c r="A190" s="10" t="inlineStr">
         <is>
-          <t>F-02</t>
+          <t>R-17</t>
         </is>
       </c>
       <c r="B190" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C190" s="12" t="inlineStr">
         <is>
-          <t>Summary tab: one line per revenue type with its accounting code</t>
+          <t>NEW: Withdraw from a NON-UCG event (refunds are handled off-platform by the host club)</t>
         </is>
       </c>
       <c r="D190" s="13" t="n"/>
@@ -9262,43 +9345,32 @@
     <row r="191">
       <c r="A191" s="10" t="inlineStr">
         <is>
-          <t>F-03</t>
+          <t>R-18</t>
         </is>
       </c>
       <c r="B191" s="11" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>R</t>
         </is>
       </c>
       <c r="C191" s="12" t="inlineStr">
         <is>
-          <t>Check the arithmetic by hand against the Stripe Dashboard for one day</t>
+          <t>NEW: Check the refund-vs-withdraw button logic across your registrations</t>
         </is>
       </c>
       <c r="D191" s="13" t="n"/>
     </row>
-    <row r="192">
-      <c r="A192" s="10" t="inlineStr">
-        <is>
-          <t>F-04</t>
-        </is>
-      </c>
-      <c r="B192" s="11" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-      <c r="C192" s="12" t="inlineStr">
-        <is>
-          <t>Date-range filter, including the smart defaults (reg-open → event+1wk per event; previous month for the aggregate)</t>
-        </is>
-      </c>
-      <c r="D192" s="13" t="n"/>
+    <row r="192" ht="20" customHeight="1">
+      <c r="A192" s="9" t="inlineStr">
+        <is>
+          <t>F  -  Finance &amp; admin (Nate + Julia as finance_admin)</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="10" t="inlineStr">
         <is>
-          <t>F-05</t>
+          <t>F-01</t>
         </is>
       </c>
       <c r="B193" s="11" t="inlineStr">
@@ -9308,7 +9380,7 @@
       </c>
       <c r="C193" s="12" t="inlineStr">
         <is>
-          <t>Per-event finance dashboard</t>
+          <t>Julia opens #/admin/finance as finance_admin, not admin</t>
         </is>
       </c>
       <c r="D193" s="13" t="n"/>
@@ -9316,7 +9388,7 @@
     <row r="194">
       <c r="A194" s="10" t="inlineStr">
         <is>
-          <t>F-06</t>
+          <t>F-02</t>
         </is>
       </c>
       <c r="B194" s="11" t="inlineStr">
@@ -9326,7 +9398,7 @@
       </c>
       <c r="C194" s="12" t="inlineStr">
         <is>
-          <t>Host payout on an event: amount owed + the calculation shown</t>
+          <t>Summary tab: one line per revenue type with its accounting code</t>
         </is>
       </c>
       <c r="D194" s="13" t="n"/>
@@ -9334,7 +9406,7 @@
     <row r="195">
       <c r="A195" s="10" t="inlineStr">
         <is>
-          <t>F-07</t>
+          <t>F-03</t>
         </is>
       </c>
       <c r="B195" s="11" t="inlineStr">
@@ -9344,7 +9416,7 @@
       </c>
       <c r="C195" s="12" t="inlineStr">
         <is>
-          <t>Enter host payment info (date, check# / PayPal / ACH)</t>
+          <t>Check the arithmetic by hand against the Stripe Dashboard for one day</t>
         </is>
       </c>
       <c r="D195" s="13" t="n"/>
@@ -9352,7 +9424,7 @@
     <row r="196">
       <c r="A196" s="10" t="inlineStr">
         <is>
-          <t>F-08</t>
+          <t>F-04</t>
         </is>
       </c>
       <c r="B196" s="11" t="inlineStr">
@@ -9362,7 +9434,7 @@
       </c>
       <c r="C196" s="12" t="inlineStr">
         <is>
-          <t>Invoices/Transactions tab</t>
+          <t>Date-range filter, including the smart defaults (reg-open → event+1wk per event; previous month for the aggregate)</t>
         </is>
       </c>
       <c r="D196" s="13" t="n"/>
@@ -9370,7 +9442,7 @@
     <row r="197">
       <c r="A197" s="10" t="inlineStr">
         <is>
-          <t>F-09</t>
+          <t>F-05</t>
         </is>
       </c>
       <c r="B197" s="11" t="inlineStr">
@@ -9380,7 +9452,7 @@
       </c>
       <c r="C197" s="12" t="inlineStr">
         <is>
-          <t>Click through from a summary line to its transactions</t>
+          <t>Per-event finance dashboard</t>
         </is>
       </c>
       <c r="D197" s="13" t="n"/>
@@ -9388,7 +9460,7 @@
     <row r="198">
       <c r="A198" s="10" t="inlineStr">
         <is>
-          <t>F-10</t>
+          <t>F-06</t>
         </is>
       </c>
       <c r="B198" s="11" t="inlineStr">
@@ -9398,7 +9470,7 @@
       </c>
       <c r="C198" s="12" t="inlineStr">
         <is>
-          <t>Export both tabs; open in Excel</t>
+          <t>Host payout on an event: amount owed + the calculation shown</t>
         </is>
       </c>
       <c r="D198" s="13" t="n"/>
@@ -9406,7 +9478,7 @@
     <row r="199">
       <c r="A199" s="10" t="inlineStr">
         <is>
-          <t>F-11</t>
+          <t>F-07</t>
         </is>
       </c>
       <c r="B199" s="11" t="inlineStr">
@@ -9416,7 +9488,7 @@
       </c>
       <c r="C199" s="12" t="inlineStr">
         <is>
-          <t>Accounting-code management: assign codes to purchase-item types</t>
+          <t>Enter host payment info (date, check# / PayPal / ACH)</t>
         </is>
       </c>
       <c r="D199" s="13" t="n"/>
@@ -9424,7 +9496,7 @@
     <row r="200">
       <c r="A200" s="10" t="inlineStr">
         <is>
-          <t>F-12</t>
+          <t>F-08</t>
         </is>
       </c>
       <c r="B200" s="11" t="inlineStr">
@@ -9434,7 +9506,7 @@
       </c>
       <c r="C200" s="12" t="inlineStr">
         <is>
-          <t>#/admin/members: search, open a profile, edit it, export a person's data, delete a person</t>
+          <t>Invoices/Transactions tab</t>
         </is>
       </c>
       <c r="D200" s="13" t="n"/>
@@ -9442,7 +9514,7 @@
     <row r="201">
       <c r="A201" s="10" t="inlineStr">
         <is>
-          <t>F-13</t>
+          <t>F-09</t>
         </is>
       </c>
       <c r="B201" s="11" t="inlineStr">
@@ -9452,7 +9524,7 @@
       </c>
       <c r="C201" s="12" t="inlineStr">
         <is>
-          <t>#/admin/clubs: create, edit, manage managers</t>
+          <t>Click through from a summary line to its transactions</t>
         </is>
       </c>
       <c r="D201" s="13" t="n"/>
@@ -9460,7 +9532,7 @@
     <row r="202">
       <c r="A202" s="10" t="inlineStr">
         <is>
-          <t>F-14</t>
+          <t>F-10</t>
         </is>
       </c>
       <c r="B202" s="11" t="inlineStr">
@@ -9470,7 +9542,7 @@
       </c>
       <c r="C202" s="12" t="inlineStr">
         <is>
-          <t>#/admin/league: seasons, levels, regions, promos, waivers, user roles</t>
+          <t>Export both tabs; open in Excel</t>
         </is>
       </c>
       <c r="D202" s="13" t="n"/>
@@ -9478,7 +9550,7 @@
     <row r="203">
       <c r="A203" s="10" t="inlineStr">
         <is>
-          <t>F-15</t>
+          <t>F-11</t>
         </is>
       </c>
       <c r="B203" s="11" t="inlineStr">
@@ -9488,7 +9560,7 @@
       </c>
       <c r="C203" s="12" t="inlineStr">
         <is>
-          <t>Grant and then revoke a role; have that person refresh</t>
+          <t>Accounting-code management: assign codes to purchase-item types</t>
         </is>
       </c>
       <c r="D203" s="13" t="n"/>
@@ -9496,7 +9568,7 @@
     <row r="204">
       <c r="A204" s="10" t="inlineStr">
         <is>
-          <t>F-16</t>
+          <t>F-12</t>
         </is>
       </c>
       <c r="B204" s="11" t="inlineStr">
@@ -9506,7 +9578,7 @@
       </c>
       <c r="C204" s="12" t="inlineStr">
         <is>
-          <t>#/admin/errors</t>
+          <t>#/admin/members: search, open a profile, edit it, export a person's data, delete a person</t>
         </is>
       </c>
       <c r="D204" s="13" t="n"/>
@@ -9514,7 +9586,7 @@
     <row r="205">
       <c r="A205" s="10" t="inlineStr">
         <is>
-          <t>F-17</t>
+          <t>F-13</t>
         </is>
       </c>
       <c r="B205" s="11" t="inlineStr">
@@ -9524,7 +9596,7 @@
       </c>
       <c r="C205" s="12" t="inlineStr">
         <is>
-          <t>Payments reconciliation tool</t>
+          <t>#/admin/clubs: create, edit, manage managers</t>
         </is>
       </c>
       <c r="D205" s="13" t="n"/>
@@ -9532,7 +9604,7 @@
     <row r="206">
       <c r="A206" s="10" t="inlineStr">
         <is>
-          <t>F-18</t>
+          <t>F-14</t>
         </is>
       </c>
       <c r="B206" s="11" t="inlineStr">
@@ -9542,32 +9614,43 @@
       </c>
       <c r="C206" s="12" t="inlineStr">
         <is>
-          <t>Manager-access request → review flow</t>
+          <t>#/admin/league: seasons, levels, regions, promos, waivers, user roles</t>
         </is>
       </c>
       <c r="D206" s="13" t="n"/>
     </row>
-    <row r="207" ht="20" customHeight="1">
-      <c r="A207" s="9" t="inlineStr">
-        <is>
-          <t>J  -  Judge &amp; meet day (2 devices required)</t>
-        </is>
-      </c>
+    <row r="207">
+      <c r="A207" s="10" t="inlineStr">
+        <is>
+          <t>F-15</t>
+        </is>
+      </c>
+      <c r="B207" s="11" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+      <c r="C207" s="12" t="inlineStr">
+        <is>
+          <t>Grant and then revoke a role; have that person refresh</t>
+        </is>
+      </c>
+      <c r="D207" s="13" t="n"/>
     </row>
     <row r="208">
       <c r="A208" s="10" t="inlineStr">
         <is>
-          <t>J-01</t>
+          <t>F-16</t>
         </is>
       </c>
       <c r="B208" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C208" s="12" t="inlineStr">
         <is>
-          <t>Admin/host: generate a judge access code for a live event</t>
+          <t>#/admin/errors</t>
         </is>
       </c>
       <c r="D208" s="13" t="n"/>
@@ -9575,17 +9658,17 @@
     <row r="209">
       <c r="A209" s="10" t="inlineStr">
         <is>
-          <t>J-02</t>
+          <t>F-17</t>
         </is>
       </c>
       <c r="B209" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C209" s="12" t="inlineStr">
         <is>
-          <t>On device 2, signed out, scan the QR with the real camera</t>
+          <t>Payments reconciliation tool</t>
         </is>
       </c>
       <c r="D209" s="13" t="n"/>
@@ -9593,43 +9676,32 @@
     <row r="210">
       <c r="A210" s="10" t="inlineStr">
         <is>
-          <t>J-03</t>
+          <t>F-18</t>
         </is>
       </c>
       <c r="B210" s="11" t="inlineStr">
         <is>
-          <t>J</t>
+          <t>F</t>
         </is>
       </c>
       <c r="C210" s="12" t="inlineStr">
         <is>
-          <t>On device 2, sign out / clear, then unlock with the 6-digit code</t>
+          <t>Manager-access request → review flow</t>
         </is>
       </c>
       <c r="D210" s="13" t="n"/>
     </row>
-    <row r="211">
-      <c r="A211" s="10" t="inlineStr">
-        <is>
-          <t>J-04</t>
-        </is>
-      </c>
-      <c r="B211" s="11" t="inlineStr">
-        <is>
-          <t>J</t>
-        </is>
-      </c>
-      <c r="C211" s="12" t="inlineStr">
-        <is>
-          <t>Enter a wrong 6-digit code</t>
-        </is>
-      </c>
-      <c r="D211" s="13" t="n"/>
+    <row r="211" ht="20" customHeight="1">
+      <c r="A211" s="9" t="inlineStr">
+        <is>
+          <t>J  -  Judge &amp; meet day (2 devices required)</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="10" t="inlineStr">
         <is>
-          <t>J-05</t>
+          <t>J-01</t>
         </is>
       </c>
       <c r="B212" s="11" t="inlineStr">
@@ -9639,7 +9711,7 @@
       </c>
       <c r="C212" s="12" t="inlineStr">
         <is>
-          <t>After being rate-limited, unlock with the URL/QR token instead</t>
+          <t>Admin/host: generate a judge access code for a live event</t>
         </is>
       </c>
       <c r="D212" s="13" t="n"/>
@@ -9647,7 +9719,7 @@
     <row r="213">
       <c r="A213" s="10" t="inlineStr">
         <is>
-          <t>J-06</t>
+          <t>J-02</t>
         </is>
       </c>
       <c r="B213" s="11" t="inlineStr">
@@ -9657,7 +9729,7 @@
       </c>
       <c r="C213" s="12" t="inlineStr">
         <is>
-          <t>After a successful unlock, try a few bad codes again</t>
+          <t>On device 2, signed out, scan the QR with the real camera</t>
         </is>
       </c>
       <c r="D213" s="13" t="n"/>
@@ -9665,7 +9737,7 @@
     <row r="214">
       <c r="A214" s="10" t="inlineStr">
         <is>
-          <t>J-07</t>
+          <t>J-03</t>
         </is>
       </c>
       <c r="B214" s="11" t="inlineStr">
@@ -9675,7 +9747,7 @@
       </c>
       <c r="C214" s="12" t="inlineStr">
         <is>
-          <t>Enter a real score from the anonymous device</t>
+          <t>On device 2, sign out / clear, then unlock with the 6-digit code</t>
         </is>
       </c>
       <c r="D214" s="13" t="n"/>
@@ -9683,7 +9755,7 @@
     <row r="215">
       <c r="A215" s="10" t="inlineStr">
         <is>
-          <t>J-08</t>
+          <t>J-04</t>
         </is>
       </c>
       <c r="B215" s="11" t="inlineStr">
@@ -9693,7 +9765,7 @@
       </c>
       <c r="C215" s="12" t="inlineStr">
         <is>
-          <t>Watch that score appear on device 1 without refreshing</t>
+          <t>Enter a wrong 6-digit code</t>
         </is>
       </c>
       <c r="D215" s="13" t="n"/>
@@ -9701,7 +9773,7 @@
     <row r="216">
       <c r="A216" s="10" t="inlineStr">
         <is>
-          <t>J-09</t>
+          <t>J-05</t>
         </is>
       </c>
       <c r="B216" s="11" t="inlineStr">
@@ -9711,7 +9783,7 @@
       </c>
       <c r="C216" s="12" t="inlineStr">
         <is>
-          <t>Use the calculator entry mode</t>
+          <t>After being rate-limited, unlock with the URL/QR token instead</t>
         </is>
       </c>
       <c r="D216" s="13" t="n"/>
@@ -9719,7 +9791,7 @@
     <row r="217">
       <c r="A217" s="10" t="inlineStr">
         <is>
-          <t>J-10</t>
+          <t>J-06</t>
         </is>
       </c>
       <c r="B217" s="11" t="inlineStr">
@@ -9729,7 +9801,7 @@
       </c>
       <c r="C217" s="12" t="inlineStr">
         <is>
-          <t>Use the simple entry mode</t>
+          <t>After a successful unlock, try a few bad codes again</t>
         </is>
       </c>
       <c r="D217" s="13" t="n"/>
@@ -9737,7 +9809,7 @@
     <row r="218">
       <c r="A218" s="10" t="inlineStr">
         <is>
-          <t>J-11</t>
+          <t>J-07</t>
         </is>
       </c>
       <c r="B218" s="11" t="inlineStr">
@@ -9747,7 +9819,7 @@
       </c>
       <c r="C218" s="12" t="inlineStr">
         <is>
-          <t>Event configured for a 2-judge panel</t>
+          <t>Enter a real score from the anonymous device</t>
         </is>
       </c>
       <c r="D218" s="13" t="n"/>
@@ -9755,7 +9827,7 @@
     <row r="219">
       <c r="A219" s="10" t="inlineStr">
         <is>
-          <t>J-12</t>
+          <t>J-08</t>
         </is>
       </c>
       <c r="B219" s="11" t="inlineStr">
@@ -9765,7 +9837,7 @@
       </c>
       <c r="C219" s="12" t="inlineStr">
         <is>
-          <t>Enter scores for each discipline you support (MAG, WAG, T&amp;T, and the specialty calculators)</t>
+          <t>Watch that score appear on device 1 without refreshing</t>
         </is>
       </c>
       <c r="D219" s="13" t="n"/>
@@ -9773,7 +9845,7 @@
     <row r="220">
       <c r="A220" s="10" t="inlineStr">
         <is>
-          <t>J-13</t>
+          <t>J-09</t>
         </is>
       </c>
       <c r="B220" s="11" t="inlineStr">
@@ -9783,7 +9855,7 @@
       </c>
       <c r="C220" s="12" t="inlineStr">
         <is>
-          <t>Edit a posted score</t>
+          <t>Use the calculator entry mode</t>
         </is>
       </c>
       <c r="D220" s="13" t="n"/>
@@ -9791,7 +9863,7 @@
     <row r="221">
       <c r="A221" s="10" t="inlineStr">
         <is>
-          <t>J-14</t>
+          <t>J-10</t>
         </is>
       </c>
       <c r="B221" s="11" t="inlineStr">
@@ -9801,7 +9873,7 @@
       </c>
       <c r="C221" s="12" t="inlineStr">
         <is>
-          <t>Open a score detail page</t>
+          <t>Use the simple entry mode</t>
         </is>
       </c>
       <c r="D221" s="13" t="n"/>
@@ -9809,7 +9881,7 @@
     <row r="222">
       <c r="A222" s="10" t="inlineStr">
         <is>
-          <t>J-15</t>
+          <t>J-11</t>
         </is>
       </c>
       <c r="B222" s="11" t="inlineStr">
@@ -9819,7 +9891,7 @@
       </c>
       <c r="C222" s="12" t="inlineStr">
         <is>
-          <t>Try score entry on a device with no unlock and no privileged account</t>
+          <t>Event configured for a 2-judge panel</t>
         </is>
       </c>
       <c r="D222" s="13" t="n"/>
@@ -9827,7 +9899,7 @@
     <row r="223">
       <c r="A223" s="10" t="inlineStr">
         <is>
-          <t>J-16</t>
+          <t>J-12</t>
         </is>
       </c>
       <c r="B223" s="11" t="inlineStr">
@@ -9837,7 +9909,7 @@
       </c>
       <c r="C223" s="12" t="inlineStr">
         <is>
-          <t>Judge on a phone in landscape, one-handed, on venue-grade wifi</t>
+          <t>Enter scores for each discipline you support (MAG, WAG, T&amp;T, and the specialty calculators)</t>
         </is>
       </c>
       <c r="D223" s="13" t="n"/>
@@ -9845,7 +9917,7 @@
     <row r="224">
       <c r="A224" s="10" t="inlineStr">
         <is>
-          <t>J-17</t>
+          <t>J-13</t>
         </is>
       </c>
       <c r="B224" s="11" t="inlineStr">
@@ -9855,32 +9927,43 @@
       </c>
       <c r="C224" s="12" t="inlineStr">
         <is>
-          <t>Turn wifi off mid-entry, then back on</t>
+          <t>Edit a posted score</t>
         </is>
       </c>
       <c r="D224" s="13" t="n"/>
     </row>
-    <row r="225" ht="20" customHeight="1">
-      <c r="A225" s="9" t="inlineStr">
-        <is>
-          <t>X  -  Public &amp; anonymous surfaces</t>
-        </is>
-      </c>
+    <row r="225">
+      <c r="A225" s="10" t="inlineStr">
+        <is>
+          <t>J-14</t>
+        </is>
+      </c>
+      <c r="B225" s="11" t="inlineStr">
+        <is>
+          <t>J</t>
+        </is>
+      </c>
+      <c r="C225" s="12" t="inlineStr">
+        <is>
+          <t>Open a score detail page</t>
+        </is>
+      </c>
+      <c r="D225" s="13" t="n"/>
     </row>
     <row r="226">
       <c r="A226" s="10" t="inlineStr">
         <is>
-          <t>X-01</t>
+          <t>J-15</t>
         </is>
       </c>
       <c r="B226" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C226" s="12" t="inlineStr">
         <is>
-          <t>Public Results index and an event's results</t>
+          <t>Try score entry on a device with no unlock and no privileged account</t>
         </is>
       </c>
       <c r="D226" s="13" t="n"/>
@@ -9888,17 +9971,17 @@
     <row r="227">
       <c r="A227" s="10" t="inlineStr">
         <is>
-          <t>X-02</t>
+          <t>J-16</t>
         </is>
       </c>
       <c r="B227" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C227" s="12" t="inlineStr">
         <is>
-          <t>Results for an event with scores across multiple sessions</t>
+          <t>Judge on a phone in both portrait and landscape, one-handed, on venue-grade wifi — every control reachable in portrait without sideways scrolling (Nate's Z-06 finding)</t>
         </is>
       </c>
       <c r="D227" s="13" t="n"/>
@@ -9906,43 +9989,32 @@
     <row r="228">
       <c r="A228" s="10" t="inlineStr">
         <is>
-          <t>X-03</t>
+          <t>J-17</t>
         </is>
       </c>
       <c r="B228" s="11" t="inlineStr">
         <is>
-          <t>X</t>
+          <t>J</t>
         </is>
       </c>
       <c r="C228" s="12" t="inlineStr">
         <is>
-          <t>Results for an event where some registrations have no session assigned</t>
+          <t>Turn wifi off mid-entry, then back on</t>
         </is>
       </c>
       <c r="D228" s="13" t="n"/>
     </row>
-    <row r="229">
-      <c r="A229" s="10" t="inlineStr">
-        <is>
-          <t>X-04</t>
-        </is>
-      </c>
-      <c r="B229" s="11" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="C229" s="12" t="inlineStr">
-        <is>
-          <t>Public Events list and an event detail page</t>
-        </is>
-      </c>
-      <c r="D229" s="13" t="n"/>
+    <row r="229" ht="20" customHeight="1">
+      <c r="A229" s="9" t="inlineStr">
+        <is>
+          <t>X  -  Public &amp; anonymous surfaces</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" s="10" t="inlineStr">
         <is>
-          <t>X-05</t>
+          <t>X-01</t>
         </is>
       </c>
       <c r="B230" s="11" t="inlineStr">
@@ -9952,7 +10024,7 @@
       </c>
       <c r="C230" s="12" t="inlineStr">
         <is>
-          <t>Home page while signed out</t>
+          <t>Public Results index and an event's results</t>
         </is>
       </c>
       <c r="D230" s="13" t="n"/>
@@ -9960,7 +10032,7 @@
     <row r="231">
       <c r="A231" s="10" t="inlineStr">
         <is>
-          <t>X-06</t>
+          <t>X-02</t>
         </is>
       </c>
       <c r="B231" s="11" t="inlineStr">
@@ -9970,7 +10042,7 @@
       </c>
       <c r="C231" s="12" t="inlineStr">
         <is>
-          <t>Try #/me, #/cart, #/admin/members while signed out</t>
+          <t>Results for an event with scores across multiple sessions</t>
         </is>
       </c>
       <c r="D231" s="13" t="n"/>
@@ -9978,7 +10050,7 @@
     <row r="232">
       <c r="A232" s="10" t="inlineStr">
         <is>
-          <t>X-07</t>
+          <t>X-03</t>
         </is>
       </c>
       <c r="B232" s="11" t="inlineStr">
@@ -9988,7 +10060,7 @@
       </c>
       <c r="C232" s="12" t="inlineStr">
         <is>
-          <t>Open a judge access URL you weren't given (guess a token)</t>
+          <t>Results for an event where some registrations have no session assigned</t>
         </is>
       </c>
       <c r="D232" s="13" t="n"/>
@@ -9996,7 +10068,7 @@
     <row r="233">
       <c r="A233" s="10" t="inlineStr">
         <is>
-          <t>X-08</t>
+          <t>X-04</t>
         </is>
       </c>
       <c r="B233" s="11" t="inlineStr">
@@ -10006,7 +10078,7 @@
       </c>
       <c r="C233" s="12" t="inlineStr">
         <is>
-          <t>Share an event link to yourself via text/Slack and open it from there</t>
+          <t>Public Events list and an event detail page</t>
         </is>
       </c>
       <c r="D233" s="13" t="n"/>
@@ -10014,7 +10086,7 @@
     <row r="234">
       <c r="A234" s="10" t="inlineStr">
         <is>
-          <t>X-09</t>
+          <t>X-05</t>
         </is>
       </c>
       <c r="B234" s="11" t="inlineStr">
@@ -10024,32 +10096,43 @@
       </c>
       <c r="C234" s="12" t="inlineStr">
         <is>
-          <t>Public pages on a phone</t>
+          <t>Home page while signed out</t>
         </is>
       </c>
       <c r="D234" s="13" t="n"/>
     </row>
-    <row r="235" ht="20" customHeight="1">
-      <c r="A235" s="9" t="inlineStr">
-        <is>
-          <t>D  -  Devices, responsive &amp; PWA</t>
-        </is>
-      </c>
+    <row r="235">
+      <c r="A235" s="10" t="inlineStr">
+        <is>
+          <t>X-06</t>
+        </is>
+      </c>
+      <c r="B235" s="11" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="C235" s="12" t="inlineStr">
+        <is>
+          <t>Try #/me, #/cart, #/admin/members while signed out</t>
+        </is>
+      </c>
+      <c r="D235" s="13" t="n"/>
     </row>
     <row r="236">
       <c r="A236" s="10" t="inlineStr">
         <is>
-          <t>D-01</t>
+          <t>X-07</t>
         </is>
       </c>
       <c r="B236" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C236" s="12" t="inlineStr">
         <is>
-          <t>Full pass on an iPhone (Safari) — sign in, register, cart, profile</t>
+          <t>Open a judge access URL you weren't given (guess a token)</t>
         </is>
       </c>
       <c r="D236" s="13" t="n"/>
@@ -10057,17 +10140,17 @@
     <row r="237">
       <c r="A237" s="10" t="inlineStr">
         <is>
-          <t>D-02</t>
+          <t>X-08</t>
         </is>
       </c>
       <c r="B237" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C237" s="12" t="inlineStr">
         <is>
-          <t>Full pass on an Android (Chrome)</t>
+          <t>Share an event link to yourself via text/Slack and open it from there</t>
         </is>
       </c>
       <c r="D237" s="13" t="n"/>
@@ -10075,43 +10158,32 @@
     <row r="238">
       <c r="A238" s="10" t="inlineStr">
         <is>
-          <t>D-03</t>
+          <t>X-09</t>
         </is>
       </c>
       <c r="B238" s="11" t="inlineStr">
         <is>
-          <t>D</t>
+          <t>X</t>
         </is>
       </c>
       <c r="C238" s="12" t="inlineStr">
         <is>
-          <t>Tablet, both orientations</t>
+          <t>Public pages on a phone</t>
         </is>
       </c>
       <c r="D238" s="13" t="n"/>
     </row>
-    <row r="239">
-      <c r="A239" s="10" t="inlineStr">
-        <is>
-          <t>D-04</t>
-        </is>
-      </c>
-      <c r="B239" s="11" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="C239" s="12" t="inlineStr">
-        <is>
-          <t>The mobile nav drawer: open, navigate, close</t>
-        </is>
-      </c>
-      <c r="D239" s="13" t="n"/>
+    <row r="239" ht="20" customHeight="1">
+      <c r="A239" s="9" t="inlineStr">
+        <is>
+          <t>D  -  Devices, responsive &amp; PWA</t>
+        </is>
+      </c>
     </row>
     <row r="240">
       <c r="A240" s="10" t="inlineStr">
         <is>
-          <t>D-05</t>
+          <t>D-01</t>
         </is>
       </c>
       <c r="B240" s="11" t="inlineStr">
@@ -10121,7 +10193,7 @@
       </c>
       <c r="C240" s="12" t="inlineStr">
         <is>
-          <t>Every modal on a phone — registration popup, refund dialog, report-a-problem</t>
+          <t>Full pass on an iPhone (Safari) — sign in, register, cart, profile</t>
         </is>
       </c>
       <c r="D240" s="13" t="n"/>
@@ -10129,7 +10201,7 @@
     <row r="241">
       <c r="A241" s="10" t="inlineStr">
         <is>
-          <t>D-06</t>
+          <t>D-02</t>
         </is>
       </c>
       <c r="B241" s="11" t="inlineStr">
@@ -10139,7 +10211,7 @@
       </c>
       <c r="C241" s="12" t="inlineStr">
         <is>
-          <t>Wide tables on a phone — admin members, finance transactions, host summary</t>
+          <t>Full pass on an Android (Chrome)</t>
         </is>
       </c>
       <c r="D241" s="13" t="n"/>
@@ -10147,7 +10219,7 @@
     <row r="242">
       <c r="A242" s="10" t="inlineStr">
         <is>
-          <t>D-07</t>
+          <t>D-03</t>
         </is>
       </c>
       <c r="B242" s="11" t="inlineStr">
@@ -10157,7 +10229,7 @@
       </c>
       <c r="C242" s="12" t="inlineStr">
         <is>
-          <t>Install the PWA ("Add to Home Screen") on iOS and Android</t>
+          <t>Tablet, both orientations</t>
         </is>
       </c>
       <c r="D242" s="13" t="n"/>
@@ -10165,7 +10237,7 @@
     <row r="243">
       <c r="A243" s="10" t="inlineStr">
         <is>
-          <t>D-08</t>
+          <t>D-04</t>
         </is>
       </c>
       <c r="B243" s="11" t="inlineStr">
@@ -10175,7 +10247,7 @@
       </c>
       <c r="C243" s="12" t="inlineStr">
         <is>
-          <t>Use the installed PWA for a full registration flow</t>
+          <t>The mobile nav drawer: open, navigate, close</t>
         </is>
       </c>
       <c r="D243" s="13" t="n"/>
@@ -10183,7 +10255,7 @@
     <row r="244">
       <c r="A244" s="10" t="inlineStr">
         <is>
-          <t>D-09</t>
+          <t>D-05</t>
         </is>
       </c>
       <c r="B244" s="11" t="inlineStr">
@@ -10193,7 +10265,7 @@
       </c>
       <c r="C244" s="12" t="inlineStr">
         <is>
-          <t>PWA update path: with the PWA installed, wait for the next deploy, then reopen it</t>
+          <t>Every modal on a phone — registration popup, refund dialog, report-a-problem</t>
         </is>
       </c>
       <c r="D244" s="13" t="n"/>
@@ -10201,7 +10273,7 @@
     <row r="245">
       <c r="A245" s="10" t="inlineStr">
         <is>
-          <t>D-10</t>
+          <t>D-06</t>
         </is>
       </c>
       <c r="B245" s="11" t="inlineStr">
@@ -10211,7 +10283,7 @@
       </c>
       <c r="C245" s="12" t="inlineStr">
         <is>
-          <t>Dark mode (OS-level) on a few pages</t>
+          <t>Wide tables on a phone — admin members, finance transactions, host summary</t>
         </is>
       </c>
       <c r="D245" s="13" t="n"/>
@@ -10219,7 +10291,7 @@
     <row r="246">
       <c r="A246" s="10" t="inlineStr">
         <is>
-          <t>D-11</t>
+          <t>D-07</t>
         </is>
       </c>
       <c r="B246" s="11" t="inlineStr">
@@ -10229,7 +10301,7 @@
       </c>
       <c r="C246" s="12" t="inlineStr">
         <is>
-          <t>Browser zoom to 200% on desktop</t>
+          <t>Install the PWA ("Add to Home Screen") on iOS and Android</t>
         </is>
       </c>
       <c r="D246" s="13" t="n"/>
@@ -10237,7 +10309,7 @@
     <row r="247">
       <c r="A247" s="10" t="inlineStr">
         <is>
-          <t>D-12</t>
+          <t>D-08</t>
         </is>
       </c>
       <c r="B247" s="11" t="inlineStr">
@@ -10247,7 +10319,7 @@
       </c>
       <c r="C247" s="12" t="inlineStr">
         <is>
-          <t>Rotate the phone mid-form</t>
+          <t>Use the installed PWA for a full registration flow</t>
         </is>
       </c>
       <c r="D247" s="13" t="n"/>
@@ -10255,7 +10327,7 @@
     <row r="248">
       <c r="A248" s="10" t="inlineStr">
         <is>
-          <t>D-13</t>
+          <t>D-09</t>
         </is>
       </c>
       <c r="B248" s="11" t="inlineStr">
@@ -10265,32 +10337,43 @@
       </c>
       <c r="C248" s="12" t="inlineStr">
         <is>
-          <t>Firefox and Edge, one flow each</t>
+          <t>PWA update path: with the PWA installed, wait for the next deploy, then reopen it</t>
         </is>
       </c>
       <c r="D248" s="13" t="n"/>
     </row>
-    <row r="249" ht="20" customHeight="1">
-      <c r="A249" s="9" t="inlineStr">
-        <is>
-          <t>Y  -  Keyboard &amp; accessibility (Nate)</t>
-        </is>
-      </c>
+    <row r="249">
+      <c r="A249" s="10" t="inlineStr">
+        <is>
+          <t>D-10</t>
+        </is>
+      </c>
+      <c r="B249" s="11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C249" s="12" t="inlineStr">
+        <is>
+          <t>Dark mode (OS-level) on a few pages</t>
+        </is>
+      </c>
+      <c r="D249" s="13" t="n"/>
     </row>
     <row r="250">
       <c r="A250" s="10" t="inlineStr">
         <is>
-          <t>Y-01</t>
+          <t>D-11</t>
         </is>
       </c>
       <c r="B250" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C250" s="12" t="inlineStr">
         <is>
-          <t>Unplug the mouse. Complete one full registration + checkout using only the keyboard</t>
+          <t>Browser zoom to 200% on desktop</t>
         </is>
       </c>
       <c r="D250" s="13" t="n"/>
@@ -10298,17 +10381,17 @@
     <row r="251">
       <c r="A251" s="10" t="inlineStr">
         <is>
-          <t>Y-02</t>
+          <t>D-12</t>
         </is>
       </c>
       <c r="B251" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C251" s="12" t="inlineStr">
         <is>
-          <t>Tab through a page — is the focus ring always visible?</t>
+          <t>Rotate the phone mid-form</t>
         </is>
       </c>
       <c r="D251" s="13" t="n"/>
@@ -10316,43 +10399,32 @@
     <row r="252">
       <c r="A252" s="10" t="inlineStr">
         <is>
-          <t>Y-03</t>
+          <t>D-13</t>
         </is>
       </c>
       <c r="B252" s="11" t="inlineStr">
         <is>
-          <t>Y</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C252" s="12" t="inlineStr">
         <is>
-          <t>Press Enter and Space on buttons — especially Details/Hide toggles, the judge score stepper, Copy-link buttons</t>
+          <t>Firefox and Edge, one flow each</t>
         </is>
       </c>
       <c r="D252" s="13" t="n"/>
     </row>
-    <row r="253">
-      <c r="A253" s="10" t="inlineStr">
-        <is>
-          <t>Y-04</t>
-        </is>
-      </c>
-      <c r="B253" s="11" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
-      <c r="C253" s="12" t="inlineStr">
-        <is>
-          <t>Open a modal, then press Tab repeatedly</t>
-        </is>
-      </c>
-      <c r="D253" s="13" t="n"/>
+    <row r="253" ht="20" customHeight="1">
+      <c r="A253" s="9" t="inlineStr">
+        <is>
+          <t>Y  -  Keyboard &amp; accessibility (Nate)</t>
+        </is>
+      </c>
     </row>
     <row r="254">
       <c r="A254" s="10" t="inlineStr">
         <is>
-          <t>Y-05</t>
+          <t>Y-01</t>
         </is>
       </c>
       <c r="B254" s="11" t="inlineStr">
@@ -10362,7 +10434,7 @@
       </c>
       <c r="C254" s="12" t="inlineStr">
         <is>
-          <t>Press Escape in a modal with unsaved changes</t>
+          <t>Unplug the mouse. Complete one full registration + checkout using only the keyboard</t>
         </is>
       </c>
       <c r="D254" s="13" t="n"/>
@@ -10370,7 +10442,7 @@
     <row r="255">
       <c r="A255" s="10" t="inlineStr">
         <is>
-          <t>Y-06</t>
+          <t>Y-02</t>
         </is>
       </c>
       <c r="B255" s="11" t="inlineStr">
@@ -10380,7 +10452,7 @@
       </c>
       <c r="C255" s="12" t="inlineStr">
         <is>
-          <t>Press Escape with two dialogs stacked</t>
+          <t>Tab through a page — is the focus ring always visible?</t>
         </is>
       </c>
       <c r="D255" s="13" t="n"/>
@@ -10388,7 +10460,7 @@
     <row r="256">
       <c r="A256" s="10" t="inlineStr">
         <is>
-          <t>Y-07</t>
+          <t>Y-03</t>
         </is>
       </c>
       <c r="B256" s="11" t="inlineStr">
@@ -10398,7 +10470,7 @@
       </c>
       <c r="C256" s="12" t="inlineStr">
         <is>
-          <t>Close a modal</t>
+          <t>Press Enter and Space on buttons — especially Details/Hide toggles, the judge score stepper, Copy-link buttons</t>
         </is>
       </c>
       <c r="D256" s="13" t="n"/>
@@ -10406,7 +10478,7 @@
     <row r="257">
       <c r="A257" s="10" t="inlineStr">
         <is>
-          <t>Y-08</t>
+          <t>Y-04</t>
         </is>
       </c>
       <c r="B257" s="11" t="inlineStr">
@@ -10416,7 +10488,7 @@
       </c>
       <c r="C257" s="12" t="inlineStr">
         <is>
-          <t>Tab order on a long form (Profile)</t>
+          <t>Open a modal, then press Tab repeatedly</t>
         </is>
       </c>
       <c r="D257" s="13" t="n"/>
@@ -10424,7 +10496,7 @@
     <row r="258">
       <c r="A258" s="10" t="inlineStr">
         <is>
-          <t>Y-09</t>
+          <t>Y-05</t>
         </is>
       </c>
       <c r="B258" s="11" t="inlineStr">
@@ -10434,7 +10506,7 @@
       </c>
       <c r="C258" s="12" t="inlineStr">
         <is>
-          <t>Squint-test every screen for low-contrast text</t>
+          <t>Press Escape in a modal with unsaved changes</t>
         </is>
       </c>
       <c r="D258" s="13" t="n"/>
@@ -10442,43 +10514,99 @@
     <row r="259">
       <c r="A259" s="10" t="inlineStr">
         <is>
+          <t>Y-06</t>
+        </is>
+      </c>
+      <c r="B259" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C259" s="12" t="inlineStr">
+        <is>
+          <t>Press Escape with two dialogs stacked</t>
+        </is>
+      </c>
+      <c r="D259" s="13" t="n"/>
+    </row>
+    <row r="260">
+      <c r="A260" s="10" t="inlineStr">
+        <is>
+          <t>Y-07</t>
+        </is>
+      </c>
+      <c r="B260" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C260" s="12" t="inlineStr">
+        <is>
+          <t>Close a modal</t>
+        </is>
+      </c>
+      <c r="D260" s="13" t="n"/>
+    </row>
+    <row r="261">
+      <c r="A261" s="10" t="inlineStr">
+        <is>
+          <t>Y-08</t>
+        </is>
+      </c>
+      <c r="B261" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C261" s="12" t="inlineStr">
+        <is>
+          <t>Tab order on a long form (Profile)</t>
+        </is>
+      </c>
+      <c r="D261" s="13" t="n"/>
+    </row>
+    <row r="262">
+      <c r="A262" s="10" t="inlineStr">
+        <is>
+          <t>Y-09</t>
+        </is>
+      </c>
+      <c r="B262" s="11" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="C262" s="12" t="inlineStr">
+        <is>
+          <t>Squint-test every screen for low-contrast text</t>
+        </is>
+      </c>
+      <c r="D262" s="13" t="n"/>
+    </row>
+    <row r="263">
+      <c r="A263" s="10" t="inlineStr">
+        <is>
           <t>Y-10</t>
         </is>
       </c>
-      <c r="B259" s="11" t="inlineStr">
+      <c r="B263" s="11" t="inlineStr">
         <is>
           <t>Y</t>
         </is>
       </c>
-      <c r="C259" s="12" t="inlineStr">
+      <c r="C263" s="12" t="inlineStr">
         <is>
           <t>If you have VoiceOver/Narrator, skim the Profile page</t>
         </is>
       </c>
-      <c r="D259" s="13" t="n"/>
-    </row>
-    <row r="260">
-      <c r="A260" s="14" t="inlineStr">
+      <c r="D263" s="13" t="n"/>
+    </row>
+    <row r="264">
+      <c r="A264" s="14" t="inlineStr">
         <is>
           <t>EXTRA  -  findings not tied to a step (use e.g. M-X-01)</t>
         </is>
       </c>
-    </row>
-    <row r="261">
-      <c r="A261" s="13" t="n"/>
-      <c r="D261" s="13" t="n"/>
-    </row>
-    <row r="262">
-      <c r="A262" s="13" t="n"/>
-      <c r="D262" s="13" t="n"/>
-    </row>
-    <row r="263">
-      <c r="A263" s="13" t="n"/>
-      <c r="D263" s="13" t="n"/>
-    </row>
-    <row r="264">
-      <c r="A264" s="13" t="n"/>
-      <c r="D264" s="13" t="n"/>
     </row>
     <row r="265">
       <c r="A265" s="13" t="n"/>
@@ -10624,39 +10752,55 @@
       <c r="A300" s="13" t="n"/>
       <c r="D300" s="13" t="n"/>
     </row>
+    <row r="301">
+      <c r="A301" s="13" t="n"/>
+      <c r="D301" s="13" t="n"/>
+    </row>
+    <row r="302">
+      <c r="A302" s="13" t="n"/>
+      <c r="D302" s="13" t="n"/>
+    </row>
+    <row r="303">
+      <c r="A303" s="13" t="n"/>
+      <c r="D303" s="13" t="n"/>
+    </row>
+    <row r="304">
+      <c r="A304" s="13" t="n"/>
+      <c r="D304" s="13" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:O300"/>
+  <autoFilter ref="A1:O304"/>
   <mergeCells count="18">
+    <mergeCell ref="A239:O239"/>
     <mergeCell ref="A81:O81"/>
-    <mergeCell ref="A235:O235"/>
     <mergeCell ref="A105:O105"/>
     <mergeCell ref="A121:O121"/>
-    <mergeCell ref="A260:O260"/>
     <mergeCell ref="A60:O60"/>
-    <mergeCell ref="A207:O207"/>
-    <mergeCell ref="A225:O225"/>
+    <mergeCell ref="A264:O264"/>
+    <mergeCell ref="A253:O253"/>
     <mergeCell ref="A94:O94"/>
     <mergeCell ref="A46:O46"/>
     <mergeCell ref="A155:O155"/>
-    <mergeCell ref="A188:O188"/>
-    <mergeCell ref="A249:O249"/>
+    <mergeCell ref="A211:O211"/>
+    <mergeCell ref="A229:O229"/>
     <mergeCell ref="A135:O135"/>
     <mergeCell ref="A173:O173"/>
     <mergeCell ref="A18:O18"/>
     <mergeCell ref="A3:O3"/>
+    <mergeCell ref="A192:O192"/>
     <mergeCell ref="A39:O39"/>
   </mergeCells>
   <dataValidations count="4">
-    <dataValidation sqref="D2:D300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="D2:D304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PASS,FAIL,MISSING,UNCLEAR,BLOCKED,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"S1,S2,S3,S4,Q,D"</formula1>
     </dataValidation>
-    <dataValidation sqref="J2:J300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N,N/A"</formula1>
     </dataValidation>
-    <dataValidation sqref="N2:N300" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="N2:N304" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Y,N"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>